<commit_message>
MSE deals & reports 2026-10-25
</commit_message>
<xml_diff>
--- a/reports/weekly_2026-W43.xlsx
+++ b/reports/weekly_2026-W43.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH21"/>
+  <dimension ref="A1:AH22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1883,35 +1883,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
+          <t>LEND</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>152</v>
+        <v>503</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3737</v>
+        <v>312819</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>63358260</v>
+        <v>54538367.62</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1.204830561888854</v>
+        <v>1.037110111674555</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>16950</v>
+        <v>174.99</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>16970</v>
+        <v>173.2</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>16983.28</v>
+        <v>171.77</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>16954.31094460798</v>
+        <v>174.3448052068449</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>16979.93</v>
+        <v>173.04</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1919,28 +1919,28 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.01972528274867269</v>
+        <v>0.7393607731268403</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>17000</v>
+        <v>175.99</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>16900</v>
+        <v>170</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>16950</v>
+        <v>175</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>28.47203639282847</v>
+        <v>34.90389010897675</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>16996.33</v>
+        <v>175.09</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>16984.19656547071</v>
+        <v>175.4634751081321</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>-0.07678128160610864</v>
+        <v>-1.896167685190464</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -1948,82 +1948,82 @@
         </is>
       </c>
       <c r="U13" s="3" t="n">
-        <v>-0.1759613458754639</v>
+        <v>-0.6375514337658039</v>
       </c>
       <c r="V13" s="3" t="n">
-        <v>0.591715976331364</v>
+        <v>3.523529411764703</v>
       </c>
       <c r="W13" s="3" t="n">
-        <v>24.58552631578947</v>
+        <v>621.9065606361829</v>
       </c>
       <c r="X13" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>347</v>
+        <v>48655</v>
       </c>
       <c r="Z13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AA13" s="3" t="n">
-        <v>9.283162132293405</v>
+        <v>15.61217427578006</v>
       </c>
       <c r="AB13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AC13" s="3" t="n">
-        <v>7.891630862337444</v>
+        <v>9.167857818623872</v>
       </c>
       <c r="AD13" s="2" t="n">
         <v>5</v>
       </c>
       <c r="AE13" s="3" t="n">
-        <v>12671652</v>
+        <v>10907673.524</v>
       </c>
       <c r="AF13" s="3" t="n">
-        <v>0.2718754016819025</v>
+        <v>1.115217649130686</v>
       </c>
       <c r="AG13" s="3" t="n">
-        <v>0.3028572472558271</v>
+        <v>0.8143309563294959</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>Мягмар</t>
+          <t>Даваа</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LEND</t>
+          <t>ERDN-1</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>503</v>
+        <v>133</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>312819</v>
+        <v>2993</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>54538367.62</v>
+        <v>50722700</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>1.037110111674555</v>
+        <v>0.9645507806167624</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>174.99</v>
+        <v>16950</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>173.2</v>
+        <v>17000</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>171.77</v>
+        <v>16986.43</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>174.3448052068449</v>
+        <v>16947.10992315402</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>173.04</v>
+        <v>16981.82</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2031,28 +2031,28 @@
         </is>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.7393607731268403</v>
+        <v>-0.02713931061442132</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>175.99</v>
+        <v>17000</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>170</v>
+        <v>16900</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>175</v>
+        <v>16950</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>34.90389010897675</v>
+        <v>35.5496157701303</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>175.09</v>
+        <v>16996.33</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>175.4634751081321</v>
+        <v>16984.19656547071</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>-1.896167685190464</v>
+        <v>-0.0582478688046284</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -2060,47 +2060,47 @@
         </is>
       </c>
       <c r="U14" s="3" t="n">
-        <v>-0.6375514337658039</v>
+        <v>-0.2183597097085266</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>3.523529411764703</v>
+        <v>0.591715976331364</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>621.9065606361829</v>
+        <v>22.50375939849624</v>
       </c>
       <c r="X14" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>48655</v>
+        <v>347</v>
       </c>
       <c r="Z14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AA14" s="3" t="n">
-        <v>15.61217427578006</v>
+        <v>11.5956958127229</v>
       </c>
       <c r="AB14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AC14" s="3" t="n">
-        <v>9.167857818623872</v>
+        <v>9.857519414384488</v>
       </c>
       <c r="AD14" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE14" s="3" t="n">
-        <v>10907673.524</v>
+        <v>10144540</v>
       </c>
       <c r="AF14" s="3" t="n">
-        <v>1.115217649130686</v>
+        <v>0.2956486127387969</v>
       </c>
       <c r="AG14" s="3" t="n">
-        <v>0.8143309563294959</v>
+        <v>0.2579590142101729</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Даваа</t>
+          <t>Мягмар</t>
         </is>
       </c>
     </row>
@@ -2779,35 +2779,35 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GAZR</t>
+          <t>ERDN</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>421</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>227365</v>
+        <v>744</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>8036258.15</v>
+        <v>12635560</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.1528187393774448</v>
+        <v>0.240279781272092</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>36.46</v>
+        <v>16990</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>35.95</v>
+        <v>16970</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>35.46</v>
+        <v>16983.28</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>35.34518571459987</v>
+        <v>16983.27956989247</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>35.91</v>
+        <v>16979.93</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2815,74 +2815,178 @@
         </is>
       </c>
       <c r="L21" s="3" t="n">
-        <v>1.269035532994911</v>
+        <v>-0.01972528274867269</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>36.76</v>
+        <v>17000</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>34.88</v>
+        <v>16970</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>35</v>
+        <v>16980</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>17.11433158137796</v>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>36.07</v>
-      </c>
-      <c r="R21" s="3" t="n">
-        <v>31.03205720263754</v>
-      </c>
+        <v>67.60752688172043</v>
+      </c>
+      <c r="Q21" s="3" t="inlineStr"/>
+      <c r="R21" s="3" t="inlineStr"/>
       <c r="S21" s="3" t="n">
-        <v>-1.691156085389522</v>
+        <v>-0.03955267804591767</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>өмнөх хаалт</t>
-        </is>
-      </c>
-      <c r="U21" s="3" t="n">
-        <v>13.89894483565126</v>
-      </c>
+          <t>нээлт</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr"/>
       <c r="V21" s="3" t="n">
-        <v>5.389908256880727</v>
+        <v>0.1767825574543247</v>
       </c>
       <c r="W21" s="3" t="n">
-        <v>540.0593824228029</v>
+        <v>39.1578947368421</v>
       </c>
       <c r="X21" s="3" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>22179</v>
+        <v>240</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AA21" s="3" t="n">
-        <v>9.664668873286505</v>
+        <v>32.2518352965757</v>
       </c>
       <c r="AB21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AC21" s="3" t="n">
+        <v>39.57086191668592</v>
+      </c>
+      <c r="AD21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE21" s="3" t="n">
+        <v>2527112</v>
+      </c>
+      <c r="AF21" s="3" t="n">
+        <v>0.1767825574543247</v>
+      </c>
+      <c r="AG21" s="3" t="inlineStr"/>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>Баасан</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GAZR</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>421</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>227365</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>8036258.15</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.1528187393774448</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>35.95</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>35.34518571459987</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>35.91</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>сүүлийн 1 цагийн жигнэсэн дундаж</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>1.269035532994911</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>36.76</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="P22" s="3" t="n">
+        <v>17.11433158137796</v>
+      </c>
+      <c r="Q22" s="3" t="n">
+        <v>36.07</v>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>31.03205720263754</v>
+      </c>
+      <c r="S22" s="3" t="n">
+        <v>-1.691156085389522</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>өмнөх хаалт</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="n">
+        <v>13.89894483565126</v>
+      </c>
+      <c r="V22" s="3" t="n">
+        <v>5.389908256880727</v>
+      </c>
+      <c r="W22" s="3" t="n">
+        <v>540.0593824228029</v>
+      </c>
+      <c r="X22" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y22" s="2" t="n">
+        <v>22179</v>
+      </c>
+      <c r="Z22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA22" s="3" t="n">
+        <v>9.664668873286505</v>
+      </c>
+      <c r="AB22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="3" t="n">
         <v>62.2180112519158</v>
       </c>
-      <c r="AD21" s="2" t="n">
+      <c r="AD22" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AE21" s="3" t="n">
+      <c r="AE22" s="3" t="n">
         <v>1607251.63</v>
       </c>
-      <c r="AF21" s="3" t="n">
+      <c r="AF22" s="3" t="n">
         <v>2.968390347867418</v>
       </c>
-      <c r="AG21" s="3" t="n">
+      <c r="AG22" s="3" t="n">
         <v>1.732943891105614</v>
       </c>
-      <c r="AH21" t="inlineStr">
+      <c r="AH22" t="inlineStr">
         <is>
           <t>Лхагва</t>
         </is>
@@ -7899,7 +8003,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
+          <t>ERDN</t>
         </is>
       </c>
       <c r="C110" s="3" t="n">
@@ -8676,77 +8780,77 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>22154186</v>
+        <v>54501050</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12671652</v>
+        <v>30486070</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-42.80244825966524</v>
+        <v>-44.0633345596094</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.5719755174033476</v>
+        <v>0.559366654403906</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>ADB</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>54501050</v>
+        <v>17026788.542</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>30486070</v>
+        <v>9369756.356000001</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-44.0633345596094</v>
+        <v>-44.97050143726392</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.559366654403906</v>
+        <v>0.5502949856273608</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>LEND</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>17026788.542</v>
+        <v>23674865.584</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>9369756.356000001</v>
+        <v>10907673.524</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>-44.97050143726392</v>
+        <v>-53.9271997752264</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.5502949856273608</v>
+        <v>0.460728002247736</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LEND</t>
+          <t>ERDN-1</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>23674865.584</v>
+        <v>22154186</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>10907673.524</v>
+        <v>10144540</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-53.9271997752264</v>
+        <v>-54.20937605200209</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.460728002247736</v>
+        <v>0.4579062394799791</v>
       </c>
     </row>
     <row r="18">
@@ -9075,7 +9179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC21"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10304,35 +10408,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
+          <t>LEND</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>152</v>
+        <v>503</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3737</v>
+        <v>312819</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>63358260</v>
+        <v>54538367.62</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1.108256772367687</v>
+        <v>0.9539800377842377</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>16950</v>
+        <v>174.99</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>16970</v>
+        <v>173.2</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>16983.28</v>
+        <v>171.77</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>16954.31094460798</v>
+        <v>174.3448052068449</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>16979.93</v>
+        <v>173.04</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -10340,28 +10444,28 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-0.01972528274867269</v>
+        <v>0.7393607731268403</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>17000</v>
+        <v>175.99</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>16900</v>
+        <v>170</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>16950</v>
+        <v>175</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>28.47203639282847</v>
+        <v>34.90389010897675</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>16996.33</v>
+        <v>175.09</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>16984.19656547071</v>
+        <v>175.4634751081321</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>-0.07678128160610864</v>
+        <v>-1.896167685190464</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -10369,65 +10473,65 @@
         </is>
       </c>
       <c r="U13" s="3" t="n">
-        <v>-0.1759613458754639</v>
+        <v>-0.6375514337658039</v>
       </c>
       <c r="V13" s="3" t="n">
-        <v>0.591715976331364</v>
+        <v>3.523529411764703</v>
       </c>
       <c r="W13" s="3" t="n">
-        <v>24.58552631578947</v>
+        <v>621.9065606361829</v>
       </c>
       <c r="X13" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>347</v>
+        <v>48655</v>
       </c>
       <c r="Z13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AA13" s="3" t="n">
-        <v>9.283162132293405</v>
+        <v>15.61217427578006</v>
       </c>
       <c r="AB13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AC13" s="3" t="n">
-        <v>7.891630862337444</v>
+        <v>9.167857818623872</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LEND</t>
+          <t>ERDN-1</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>503</v>
+        <v>133</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>312819</v>
+        <v>2993</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>54538367.62</v>
+        <v>50722700</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.9539800377842377</v>
+        <v>0.8872367357906367</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>174.99</v>
+        <v>16950</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>173.2</v>
+        <v>17000</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>171.77</v>
+        <v>16986.43</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>174.3448052068449</v>
+        <v>16947.10992315402</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>173.04</v>
+        <v>16981.82</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -10435,28 +10539,28 @@
         </is>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.7393607731268403</v>
+        <v>-0.02713931061442132</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>175.99</v>
+        <v>17000</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>170</v>
+        <v>16900</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>175</v>
+        <v>16950</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>34.90389010897675</v>
+        <v>35.5496157701303</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>175.09</v>
+        <v>16996.33</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>175.4634751081321</v>
+        <v>16984.19656547071</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>-1.896167685190464</v>
+        <v>-0.0582478688046284</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -10464,31 +10568,31 @@
         </is>
       </c>
       <c r="U14" s="3" t="n">
-        <v>-0.6375514337658039</v>
+        <v>-0.2183597097085266</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>3.523529411764703</v>
+        <v>0.591715976331364</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>621.9065606361829</v>
+        <v>22.50375939849624</v>
       </c>
       <c r="X14" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>48655</v>
+        <v>347</v>
       </c>
       <c r="Z14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AA14" s="3" t="n">
-        <v>15.61217427578006</v>
+        <v>11.5956958127229</v>
       </c>
       <c r="AB14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AC14" s="3" t="n">
-        <v>9.167857818623872</v>
+        <v>9.857519414384488</v>
       </c>
     </row>
     <row r="15">
@@ -11064,35 +11168,35 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GAZR</t>
+          <t>ERDN</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>421</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>227365</v>
+        <v>744</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>8036258.15</v>
+        <v>12635560</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.140569477748166</v>
+        <v>0.22102003657705</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>36.46</v>
+        <v>16990</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>35.95</v>
+        <v>16970</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>35.46</v>
+        <v>16983.28</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>35.34518571459987</v>
+        <v>16983.27956989247</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>35.91</v>
+        <v>16979.93</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -11100,59 +11204,148 @@
         </is>
       </c>
       <c r="L21" s="3" t="n">
-        <v>1.269035532994911</v>
+        <v>-0.01972528274867269</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>36.76</v>
+        <v>17000</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>34.88</v>
+        <v>16970</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>35</v>
+        <v>16980</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>17.11433158137796</v>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>36.07</v>
-      </c>
-      <c r="R21" s="3" t="n">
-        <v>31.03205720263754</v>
-      </c>
+        <v>67.60752688172043</v>
+      </c>
+      <c r="Q21" s="3" t="inlineStr"/>
+      <c r="R21" s="3" t="inlineStr"/>
       <c r="S21" s="3" t="n">
-        <v>-1.691156085389522</v>
+        <v>-0.03955267804591767</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>өмнөх хаалт</t>
-        </is>
-      </c>
-      <c r="U21" s="3" t="n">
-        <v>13.89894483565126</v>
-      </c>
+          <t>нээлт</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr"/>
       <c r="V21" s="3" t="n">
-        <v>5.389908256880727</v>
+        <v>0.1767825574543247</v>
       </c>
       <c r="W21" s="3" t="n">
-        <v>540.0593824228029</v>
+        <v>39.1578947368421</v>
       </c>
       <c r="X21" s="3" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>22179</v>
+        <v>240</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AA21" s="3" t="n">
-        <v>9.664668873286505</v>
+        <v>32.2518352965757</v>
       </c>
       <c r="AB21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AC21" s="3" t="n">
+        <v>39.57086191668592</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GAZR</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>421</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>227365</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>8036258.15</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.140569477748166</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>35.95</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>35.34518571459987</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>35.91</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>сүүлийн 1 цагийн жигнэсэн дундаж</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>1.269035532994911</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>36.76</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="P22" s="3" t="n">
+        <v>17.11433158137796</v>
+      </c>
+      <c r="Q22" s="3" t="n">
+        <v>36.07</v>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>31.03205720263754</v>
+      </c>
+      <c r="S22" s="3" t="n">
+        <v>-1.691156085389522</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>өмнөх хаалт</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="n">
+        <v>13.89894483565126</v>
+      </c>
+      <c r="V22" s="3" t="n">
+        <v>5.389908256880727</v>
+      </c>
+      <c r="W22" s="3" t="n">
+        <v>540.0593824228029</v>
+      </c>
+      <c r="X22" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y22" s="2" t="n">
+        <v>22179</v>
+      </c>
+      <c r="Z22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA22" s="3" t="n">
+        <v>9.664668873286505</v>
+      </c>
+      <c r="AB22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="3" t="n">
         <v>62.2180112519158</v>
       </c>
     </row>
@@ -11385,10 +11578,10 @@
         <v>801621237.17</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-0.4985969762007508</v>
+        <v>-0.5238635197458976</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-1.102747544745537</v>
+        <v>-1.120111183613114</v>
       </c>
     </row>
   </sheetData>
@@ -11402,7 +11595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11729,51 +11922,51 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
+          <t>LEND</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>11555680</v>
+        <v>25402662.53</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>22257460</v>
+        <v>5894246.399999999</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>4356590</v>
+        <v>13191728.96</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>12552970</v>
+        <v>2865214.38</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>12635560</v>
+        <v>7184515.35</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>63358260</v>
+        <v>54538367.62</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LEND</t>
+          <t>ERDN-1</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>25402662.53</v>
+        <v>11555680</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>5894246.399999999</v>
+        <v>22257460</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13191728.96</v>
+        <v>4356590</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>2865214.38</v>
+        <v>12552970</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>7184515.35</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>54538367.62</v>
+        <v>50722700</v>
       </c>
     </row>
     <row r="15">
@@ -11929,25 +12122,50 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>ERDN</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>12635560</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>12635560</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>GAZR</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="3" t="n">
         <v>688678.64</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C22" s="3" t="n">
         <v>1865844.14</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D22" s="3" t="n">
         <v>3107496</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E22" s="3" t="n">
         <v>1166178</v>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F22" s="3" t="n">
         <v>1208061.37</v>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="G22" s="3" t="n">
         <v>8036258.149999999</v>
       </c>
     </row>
@@ -11962,7 +12180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12096,21 +12314,13 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>16900</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>16900</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>16990</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>17000</v>
-      </c>
+          <t>ERDN</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="n">
         <v>16970</v>
       </c>
@@ -12118,330 +12328,350 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GAZR</t>
+          <t>ERDN-1</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>35.99</v>
+        <v>16900</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>35.98</v>
+        <v>16900</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>35.96</v>
+        <v>16990</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>35.95</v>
-      </c>
+        <v>17000</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GLMT</t>
+          <t>GAZR</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1300</v>
+        <v>35.99</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1305</v>
+        <v>35.98</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1306</v>
+        <v>35.96</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1289</v>
+        <v>35.2</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1289</v>
+        <v>35.95</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>GLMT</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>7810</v>
+        <v>1300</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>7800</v>
+        <v>1305</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7700</v>
+        <v>1306</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>7700</v>
+        <v>1289</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>7700</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KHAN</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>2086</v>
+        <v>7810</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>2085</v>
+        <v>7800</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2085</v>
+        <v>7700</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2085</v>
+        <v>7700</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>2084</v>
+        <v>7700</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LEND</t>
+          <t>KHAN</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>174.5</v>
+        <v>2086</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>175.88</v>
+        <v>2085</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>173.99</v>
+        <v>2085</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>172.99</v>
+        <v>2085</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>173.2</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MFC</t>
+          <t>LEND</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>79.8</v>
+        <v>174.5</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>77</v>
+        <v>175.88</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>78.98999999999999</v>
+        <v>173.99</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>78.98</v>
+        <v>172.99</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>78.97</v>
+        <v>173.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MFG</t>
+          <t>MFC</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>1310</v>
+        <v>79.8</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1305</v>
+        <v>77</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>1337</v>
+        <v>78.98999999999999</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1339</v>
+        <v>78.98</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1339</v>
+        <v>78.97</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MNDL</t>
+          <t>MFG</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>89</v>
+        <v>1310</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>88.45999999999999</v>
+        <v>1305</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>88.95</v>
+        <v>1337</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>88</v>
+        <v>1339</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>90.41</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>MNDL</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>374.5</v>
+        <v>89</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>398.39</v>
+        <v>88.45999999999999</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>395</v>
+        <v>88.95</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>396.78</v>
+        <v>88</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>399.98</v>
+        <v>90.41</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>QPAY</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>518</v>
+        <v>374.5</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>524.86</v>
+        <v>398.39</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>524</v>
+        <v>395</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>519.95</v>
+        <v>396.78</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>515</v>
+        <v>399.98</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SBM</t>
+          <t>QPAY</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>589.79</v>
+        <v>518</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>589</v>
+        <v>524.86</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>588.1</v>
+        <v>524</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>589</v>
+        <v>519.95</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>589</v>
+        <v>515</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TDB</t>
+          <t>SBM</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>12300</v>
+        <v>589.79</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>11300</v>
+        <v>589</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>11900</v>
+        <v>588.1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>12480</v>
+        <v>589</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>12470</v>
+        <v>589</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>TDB</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>59500</v>
+        <v>12300</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>59500</v>
+        <v>11300</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>59650</v>
+        <v>11900</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>59500</v>
+        <v>12480</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>59700</v>
+        <v>12470</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TUM</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>512</v>
+        <v>59500</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>509</v>
+        <v>59500</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>507.88</v>
+        <v>59650</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>507</v>
+        <v>59500</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>503</v>
+        <v>59700</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>TUM</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>512</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>509</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>507.88</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>507</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>XAC</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="3" t="n">
         <v>1625</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C22" s="3" t="n">
         <v>1630</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D22" s="3" t="n">
         <v>1620</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E22" s="3" t="n">
         <v>1605</v>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F22" s="3" t="n">
         <v>1600</v>
       </c>
     </row>
@@ -12456,7 +12686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:V22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12480,6 +12710,7 @@
     <col width="8" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
     <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12510,80 +12741,85 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>ERDN</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>ERDN-1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>GAZR</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>GLMT</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>INV</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>KHAN</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>LEND</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MFC</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>MFG</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>MNDL</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MSE</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>QPAY</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>SBM</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>TDB</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>TTL</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>TUM</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>XAC</t>
         </is>
@@ -12607,52 +12843,53 @@
       <c r="E2" s="3" t="n">
         <v>0.79</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>0.83</v>
-      </c>
+      <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>-0.01</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>-0.03</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>-0.87</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>-0.9</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>0.97</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>0.21</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="P2" s="3" t="n">
         <v>-0.83</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>-0.41</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="R2" s="3" t="n">
         <v>-0.23</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="S2" s="3" t="n">
         <v>0.79</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="T2" s="3" t="n">
         <v>0.41</v>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="U2" s="3" t="n">
         <v>0.53</v>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="V2" s="3" t="n">
         <v>-0.6</v>
       </c>
     </row>
@@ -12674,52 +12911,53 @@
       <c r="E3" s="3" t="n">
         <v>-0.99</v>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>-0.51</v>
-      </c>
+      <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>-0.63</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>-0.6</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>0.75</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="K3" s="3" t="n">
         <v>-0.02</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>0.38</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>-0.62</v>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>-0.73</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="O3" s="3" t="n">
         <v>-0.66</v>
       </c>
-      <c r="O3" s="3" t="n">
+      <c r="P3" s="3" t="n">
         <v>0.44</v>
       </c>
-      <c r="P3" s="3" t="n">
+      <c r="Q3" s="3" t="n">
         <v>0.13</v>
       </c>
-      <c r="Q3" s="3" t="n">
+      <c r="R3" s="3" t="n">
         <v>0.66</v>
       </c>
-      <c r="R3" s="3" t="n">
+      <c r="S3" s="3" t="n">
         <v>-0.24</v>
       </c>
-      <c r="S3" s="3" t="n">
+      <c r="T3" s="3" t="n">
         <v>-0.91</v>
       </c>
-      <c r="T3" s="3" t="n">
+      <c r="U3" s="3" t="n">
         <v>0.15</v>
       </c>
-      <c r="U3" s="3" t="n">
+      <c r="V3" s="3" t="n">
         <v>-0.02</v>
       </c>
     </row>
@@ -12741,52 +12979,53 @@
       <c r="E4" s="3" t="n">
         <v>-0.3</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>0.62</v>
-      </c>
+      <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>-0.83</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="I4" s="3" t="n">
         <v>-0.19</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>-0.38</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="K4" s="3" t="n">
         <v>0.58</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="L4" s="3" t="n">
         <v>-0.25</v>
       </c>
-      <c r="L4" s="3" t="n">
+      <c r="M4" s="3" t="n">
         <v>-0.06</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="N4" s="3" t="n">
         <v>0.29</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="O4" s="3" t="n">
         <v>-0.92</v>
       </c>
-      <c r="O4" s="3" t="n">
+      <c r="P4" s="3" t="n">
         <v>0.19</v>
       </c>
-      <c r="P4" s="3" t="n">
+      <c r="Q4" s="3" t="n">
         <v>0.52</v>
       </c>
-      <c r="Q4" s="3" t="n">
+      <c r="R4" s="3" t="n">
         <v>-0.16</v>
       </c>
-      <c r="R4" s="3" t="n">
+      <c r="S4" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="S4" s="3" t="n">
+      <c r="T4" s="3" t="n">
         <v>-0.63</v>
       </c>
-      <c r="T4" s="3" t="n">
+      <c r="U4" s="3" t="n">
         <v>0.78</v>
       </c>
-      <c r="U4" s="3" t="n">
+      <c r="V4" s="3" t="n">
         <v>-0.09</v>
       </c>
     </row>
@@ -12808,1124 +13047,1169 @@
       <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>0.54</v>
-      </c>
+      <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H5" s="3" t="n">
         <v>0.58</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="I5" s="3" t="n">
         <v>0.51</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>-0.77</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>0.11</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="L5" s="3" t="n">
         <v>-0.47</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="M5" s="3" t="n">
         <v>0.71</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="N5" s="3" t="n">
         <v>0.78</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="O5" s="3" t="n">
         <v>0.65</v>
       </c>
-      <c r="O5" s="3" t="n">
+      <c r="P5" s="3" t="n">
         <v>-0.54</v>
       </c>
-      <c r="P5" s="3" t="n">
+      <c r="Q5" s="3" t="n">
         <v>-0.22</v>
       </c>
-      <c r="Q5" s="3" t="n">
+      <c r="R5" s="3" t="n">
         <v>-0.58</v>
       </c>
-      <c r="R5" s="3" t="n">
+      <c r="S5" s="3" t="n">
         <v>0.35</v>
       </c>
-      <c r="S5" s="3" t="n">
+      <c r="T5" s="3" t="n">
         <v>0.88</v>
       </c>
-      <c r="T5" s="3" t="n">
+      <c r="U5" s="3" t="n">
         <v>-0.08</v>
       </c>
-      <c r="U5" s="3" t="n">
+      <c r="V5" s="3" t="n">
         <v>-0.09</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ERDN-1</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>-0.95</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>-0.74</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>-0.27</v>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>-0.44</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>-0.45</v>
-      </c>
-      <c r="R6" s="3" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="S6" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="U6" s="3" t="n">
-        <v>-0.35</v>
-      </c>
+          <t>ERDN</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="3" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" s="3" t="inlineStr"/>
+      <c r="S6" s="3" t="inlineStr"/>
+      <c r="T6" s="3" t="inlineStr"/>
+      <c r="U6" s="3" t="inlineStr"/>
+      <c r="V6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GAZR</t>
+          <t>ERDN-1</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>-0.01</v>
+        <v>0.93</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>-0.63</v>
+        <v>-0.7</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>-0.83</v>
+        <v>0.38</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>-0.33</v>
-      </c>
+        <v>0.74</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.7</v>
+        <v>-0.11</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>-0.71</v>
+        <v>-0.98</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.35</v>
+        <v>0.66</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-0</v>
+        <v>-0.79</v>
       </c>
       <c r="M7" s="3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="Q7" s="3" t="n">
         <v>-0.06</v>
       </c>
-      <c r="N7" s="3" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>-0.08</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>-0.43</v>
-      </c>
       <c r="R7" s="3" t="n">
-        <v>-0.32</v>
+        <v>-0.48</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>0.9</v>
+        <v>0.58</v>
       </c>
       <c r="T7" s="3" t="n">
-        <v>-0.86</v>
+        <v>0.34</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>0.47</v>
+        <v>0.59</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>-0.38</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GLMT</t>
+          <t>GAZR</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>-0.03</v>
+        <v>-0.01</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.63</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.83</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>0.08</v>
-      </c>
+        <v>0.58</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="n">
-        <v>0.7</v>
+        <v>-0.11</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I8" s="3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="S8" s="3" t="n">
         <v>-0.32</v>
       </c>
-      <c r="J8" s="3" t="n">
-        <v>-0.62</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>-0.24</v>
-      </c>
-      <c r="M8" s="3" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="N8" s="3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="O8" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q8" s="3" t="n">
-        <v>-0.92</v>
-      </c>
-      <c r="R8" s="3" t="n">
-        <v>-0.62</v>
-      </c>
-      <c r="S8" s="3" t="n">
-        <v>0.7</v>
-      </c>
       <c r="T8" s="3" t="n">
-        <v>-0.59</v>
+        <v>0.9</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>-0.86</v>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>0.47</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INV</t>
+          <t>GLMT</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>-0.87</v>
+        <v>-0.03</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.75</v>
+        <v>-0.6</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.38</v>
+        <v>-0.19</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>-0.95</v>
-      </c>
+        <v>0.51</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="n">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-0.32</v>
+        <v>0.7</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>-0.54</v>
+        <v>-0.32</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0.67</v>
+        <v>-0.62</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-0.68</v>
+        <v>0.45</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>-0.96</v>
+        <v>-0.24</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.11</v>
       </c>
       <c r="O9" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P9" s="3" t="n">
         <v>0.45</v>
       </c>
-      <c r="P9" s="3" t="n">
-        <v>-0.08</v>
-      </c>
       <c r="Q9" s="3" t="n">
-        <v>0.63</v>
+        <v>0.6</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>-0.43</v>
+        <v>-0.92</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>-0.41</v>
+        <v>-0.62</v>
       </c>
       <c r="T9" s="3" t="n">
-        <v>-0.48</v>
+        <v>0.7</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>0.21</v>
+        <v>-0.59</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KHAN</t>
+          <t>INV</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>-0.87</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.75</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.58</v>
+        <v>-0.38</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>0.73</v>
-      </c>
+        <v>-0.77</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="n">
-        <v>-0.71</v>
+        <v>-0.98</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>-0.62</v>
+        <v>0.02</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>-0.54</v>
+        <v>-0.32</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>-0.91</v>
+        <v>-0.54</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.67</v>
+        <v>-0.68</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>-0.45</v>
+        <v>-0.96</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>-0.68</v>
+        <v>-0.02</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>-0.37</v>
+        <v>0.45</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.27</v>
+        <v>-0.08</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>-0.37</v>
+        <v>-0.43</v>
       </c>
       <c r="T10" s="3" t="n">
-        <v>0.96</v>
+        <v>-0.41</v>
       </c>
       <c r="U10" s="3" t="n">
-        <v>-0.84</v>
+        <v>-0.48</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>0.21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LEND</t>
+          <t>KHAN</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>-0.9</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.38</v>
+        <v>-0.02</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.25</v>
+        <v>0.58</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>-0.74</v>
-      </c>
+        <v>0.11</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="n">
-        <v>0.35</v>
+        <v>0.66</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.45</v>
+        <v>-0.71</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.67</v>
+        <v>-0.62</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-0.91</v>
+        <v>-0.54</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.91</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-0.83</v>
+        <v>0.7</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.04</v>
+        <v>0.67</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.9</v>
+        <v>-0.45</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.57</v>
+        <v>-0.68</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.37</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>-0.96</v>
+        <v>0.27</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>-0.04</v>
+        <v>0.85</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>-0.76</v>
+        <v>-0.37</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>0.87</v>
+        <v>0.96</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>-0.84</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MFC</t>
+          <t>LEND</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.95</v>
+        <v>-0.9</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>-0.62</v>
+        <v>0.38</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.06</v>
+        <v>-0.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>0.65</v>
-      </c>
+        <v>-0.47</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="n">
-        <v>-0</v>
+        <v>-0.79</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>-0.24</v>
+        <v>0.35</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>-0.68</v>
+        <v>0.45</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.91</v>
       </c>
       <c r="L12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.85</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.31</v>
+        <v>-0.83</v>
       </c>
       <c r="O12" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="S12" s="3" t="n">
         <v>-0.96</v>
       </c>
-      <c r="P12" s="3" t="n">
-        <v>-0.67</v>
-      </c>
-      <c r="Q12" s="3" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="R12" s="3" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="S12" s="3" t="n">
-        <v>0.37</v>
-      </c>
       <c r="T12" s="3" t="n">
-        <v>0.49</v>
+        <v>-0.04</v>
       </c>
       <c r="U12" s="3" t="n">
         <v>-0.76</v>
       </c>
+      <c r="V12" s="3" t="n">
+        <v>0.87</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MFG</t>
+          <t>MFC</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>-0.73</v>
+        <v>-0.62</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.29</v>
+        <v>-0.06</v>
       </c>
       <c r="E13" s="3" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="n">
         <v>0.78</v>
       </c>
-      <c r="F13" s="3" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>-0.06</v>
-      </c>
       <c r="H13" s="3" t="n">
-        <v>0.11</v>
+        <v>-0</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-0.96</v>
+        <v>-0.24</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.67</v>
+        <v>-0.68</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-0.83</v>
+        <v>0.7</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0.85</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.08</v>
+        <v>0.85</v>
       </c>
       <c r="O13" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="P13" s="3" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="Q13" s="3" t="n">
         <v>-0.67</v>
       </c>
-      <c r="P13" s="3" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="Q13" s="3" t="n">
-        <v>-0.41</v>
-      </c>
       <c r="R13" s="3" t="n">
-        <v>0.65</v>
+        <v>0.04</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>0.38</v>
+        <v>0.91</v>
       </c>
       <c r="T13" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.37</v>
       </c>
       <c r="U13" s="3" t="n">
-        <v>-0.45</v>
+        <v>0.49</v>
+      </c>
+      <c r="V13" s="3" t="n">
+        <v>-0.76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MNDL</t>
+          <t>MFG</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.21</v>
+        <v>0.97</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>-0.66</v>
+        <v>-0.73</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.92</v>
+        <v>0.29</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>-0.27</v>
-      </c>
+        <v>0.78</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="n">
-        <v>0.92</v>
+        <v>0.99</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.4</v>
+        <v>-0.06</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.11</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>-0.45</v>
+        <v>-0.96</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0.04</v>
+        <v>0.67</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.31</v>
+        <v>-0.83</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.08</v>
+        <v>0.85</v>
       </c>
       <c r="N14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>-0.33</v>
+        <v>0.08</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>-0.46</v>
+        <v>-0.67</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.18</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.05</v>
+        <v>-0.41</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0.88</v>
+        <v>0.65</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>-0.68</v>
+        <v>0.38</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.09</v>
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="V14" s="3" t="n">
+        <v>-0.45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>MNDL</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>-0.83</v>
+        <v>0.21</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.44</v>
+        <v>-0.66</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.19</v>
+        <v>-0.92</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>-0.44</v>
-      </c>
+        <v>0.65</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="L15" s="3" t="n">
         <v>0.04</v>
       </c>
-      <c r="H15" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>-0.68</v>
-      </c>
-      <c r="K15" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="L15" s="3" t="n">
-        <v>-0.96</v>
-      </c>
       <c r="M15" s="3" t="n">
-        <v>-0.67</v>
+        <v>0.31</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>-0.33</v>
+        <v>0.08</v>
       </c>
       <c r="O15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>0.85</v>
+        <v>-0.33</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>-0.31</v>
+        <v>-0.46</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>-0.96</v>
+        <v>-0.16</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>-0.25</v>
+        <v>0.05</v>
       </c>
       <c r="T15" s="3" t="n">
-        <v>-0.45</v>
+        <v>0.88</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>0.88</v>
+        <v>-0.68</v>
+      </c>
+      <c r="V15" s="3" t="n">
+        <v>0.09</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>QPAY</t>
+          <t>MSE</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>-0.41</v>
+        <v>-0.83</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.13</v>
+        <v>0.44</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.52</v>
+        <v>0.19</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.22</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>0.1</v>
-      </c>
+        <v>-0.54</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="n">
-        <v>-0.08</v>
+        <v>-0.58</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.6</v>
+        <v>0.04</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-0.08</v>
+        <v>0.45</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-0.37</v>
+        <v>0.45</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.57</v>
+        <v>-0.68</v>
       </c>
       <c r="L16" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="N16" s="3" t="n">
         <v>-0.67</v>
       </c>
-      <c r="M16" s="3" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="N16" s="3" t="n">
-        <v>-0.46</v>
-      </c>
       <c r="O16" s="3" t="n">
-        <v>0.85</v>
+        <v>-0.33</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>-0.66</v>
+        <v>0.85</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>-0.78</v>
+        <v>-0.31</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>-0.15</v>
+        <v>-0.96</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>-0.11</v>
+        <v>-0.25</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.8</v>
+        <v>-0.45</v>
+      </c>
+      <c r="V16" s="3" t="n">
+        <v>0.88</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SBM</t>
+          <t>QPAY</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>-0.23</v>
+        <v>-0.41</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0.66</v>
+        <v>0.13</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.16</v>
+        <v>0.52</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.58</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>-0.45</v>
-      </c>
+        <v>-0.22</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="3" t="n">
-        <v>-0.43</v>
+        <v>-0.06</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.92</v>
+        <v>-0.08</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0.63</v>
+        <v>0.6</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.27</v>
+        <v>-0.08</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.37</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.04</v>
+        <v>0.57</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-0.41</v>
+        <v>-0.67</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.18</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>-0.31</v>
+        <v>-0.46</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>-0.66</v>
+        <v>0.85</v>
       </c>
       <c r="Q17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>0.41</v>
+        <v>-0.66</v>
       </c>
       <c r="S17" s="3" t="n">
-        <v>-0.58</v>
+        <v>-0.78</v>
       </c>
       <c r="T17" s="3" t="n">
-        <v>0.21</v>
+        <v>-0.15</v>
       </c>
       <c r="U17" s="3" t="n">
-        <v>-0.63</v>
+        <v>-0.11</v>
+      </c>
+      <c r="V17" s="3" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TDB</t>
+          <t>SBM</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.79</v>
+        <v>-0.23</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>-0.24</v>
+        <v>0.66</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.06</v>
+        <v>-0.16</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>0.52</v>
-      </c>
+        <v>-0.58</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="n">
-        <v>-0.32</v>
+        <v>-0.48</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>-0.62</v>
+        <v>-0.43</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-0.43</v>
+        <v>-0.92</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-0.96</v>
+        <v>0.27</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.91</v>
+        <v>-0.16</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.65</v>
+        <v>0.04</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.05</v>
+        <v>-0.41</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>-0.96</v>
+        <v>-0.16</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>-0.78</v>
+        <v>-0.31</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.41</v>
+        <v>-0.66</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.41</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>0.66</v>
+        <v>-0.58</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>-0.96</v>
+        <v>0.21</v>
+      </c>
+      <c r="V18" s="3" t="n">
+        <v>-0.63</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TTL</t>
+          <t>TDB</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P19" s="3" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>-0.78</v>
+      </c>
+      <c r="R19" s="3" t="n">
         <v>0.41</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>-0.91</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>-0.63</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>-0.37</v>
-      </c>
-      <c r="K19" s="3" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="L19" s="3" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="M19" s="3" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="O19" s="3" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="P19" s="3" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="Q19" s="3" t="n">
-        <v>-0.58</v>
-      </c>
-      <c r="R19" s="3" t="n">
-        <v>-0.02</v>
       </c>
       <c r="S19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>-0.54</v>
+        <v>-0.02</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>0.25</v>
+        <v>0.66</v>
+      </c>
+      <c r="V19" s="3" t="n">
+        <v>-0.96</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TUM</t>
+          <t>TTL</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.53</v>
+        <v>0.41</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.15</v>
+        <v>-0.91</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.78</v>
+        <v>-0.63</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>-0.08</v>
-      </c>
-      <c r="F20" s="3" t="n">
-        <v>0.73</v>
-      </c>
+        <v>0.88</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="n">
-        <v>-0.86</v>
+        <v>0.34</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>-0.59</v>
+        <v>0.9</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-0.48</v>
+        <v>0.7</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.96</v>
+        <v>-0.41</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>-0.76</v>
+        <v>-0.37</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.49</v>
+        <v>-0.04</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.37</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>-0.68</v>
+        <v>0.38</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>-0.45</v>
+        <v>0.88</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>-0.11</v>
+        <v>-0.25</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.21</v>
+        <v>-0.15</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.66</v>
+        <v>-0.58</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>-0.54</v>
+        <v>-0.02</v>
       </c>
       <c r="T20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.54</v>
+      </c>
+      <c r="V20" s="3" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>XAC</t>
+          <t>TUM</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>-0.6</v>
+        <v>0.53</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.15</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.09</v>
+        <v>0.78</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>-0.35</v>
-      </c>
+        <v>-0.08</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="n">
-        <v>0.47</v>
+        <v>0.59</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>-0.86</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.21</v>
+        <v>-0.59</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>-0.84</v>
+        <v>-0.48</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.87</v>
+        <v>0.96</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>-0.76</v>
       </c>
       <c r="M21" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="P21" s="3" t="n">
         <v>-0.45</v>
       </c>
-      <c r="N21" s="3" t="n">
+      <c r="Q21" s="3" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="S21" s="3" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="T21" s="3" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="U21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V21" s="3" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>XAC</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>-0.84</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="O22" s="3" t="n">
         <v>0.09</v>
       </c>
-      <c r="O21" s="3" t="n">
+      <c r="P22" s="3" t="n">
         <v>0.88</v>
       </c>
-      <c r="P21" s="3" t="n">
+      <c r="Q22" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="Q21" s="3" t="n">
+      <c r="R22" s="3" t="n">
         <v>-0.63</v>
       </c>
-      <c r="R21" s="3" t="n">
+      <c r="S22" s="3" t="n">
         <v>-0.96</v>
       </c>
-      <c r="S21" s="3" t="n">
+      <c r="T22" s="3" t="n">
         <v>0.25</v>
       </c>
-      <c r="T21" s="3" t="n">
+      <c r="U22" s="3" t="n">
         <v>-0.6899999999999999</v>
       </c>
-      <c r="U21" s="3" t="n">
+      <c r="V22" s="3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13940,7 +14224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14630,7 +14914,7 @@
         <v>0.1028812730210142</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>9.283162132293405</v>
+        <v>11.5956958127229</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -14638,35 +14922,35 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SBM</t>
+          <t>ERDN</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>46314.53350694444</v>
+        <v>46318.49207175926</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>5900</v>
+        <v>240</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>587</v>
+        <v>16980</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>587</v>
+        <v>16980</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>587</v>
+        <v>16980</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>3463300</v>
+        <v>4075200</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0.06057972046172053</v>
+        <v>0.07128301816926154</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>14.2197799490921</v>
+        <v>32.2518352965757</v>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -14674,35 +14958,35 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MFC</t>
+          <t>SBM</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>46314.4574074074</v>
+        <v>46314.53350694444</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>33253</v>
+        <v>5900</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>78</v>
+        <v>587</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>78</v>
+        <v>587</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>78</v>
+        <v>587</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>2593734</v>
+        <v>3463300</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0.04536935312333908</v>
+        <v>0.06057972046172053</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>11.36594910080954</v>
+        <v>14.2197799490921</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
@@ -14710,38 +14994,74 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GAZR</t>
+          <t>MFC</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>46316.47109953704</v>
+        <v>46314.4574074074</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>22179</v>
+        <v>33253</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>35.01860949546869</v>
+        <v>78</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>35.1</v>
+        <v>78</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>776677.74</v>
+        <v>2593734</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.0135855745612684</v>
+        <v>0.04536935312333908</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>9.664668873286507</v>
+        <v>11.36594910080954</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GAZR</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>46316.47109953704</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>22179</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>35.01860949546869</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>776677.74</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.0135855745612684</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>9.664668873286507</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>